<commit_message>
Added night shift extra cost calculation
</commit_message>
<xml_diff>
--- a/trip.xlsx
+++ b/trip.xlsx
@@ -1,119 +1,51 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python_Project\Python Learn\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C440738F-6083-4B1E-8048-14931E5C7B45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{311BBF47-CFB3-4EF9-A906-C050A2131109}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="swami" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="shekhar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="16">
-  <si>
-    <t>trip ID</t>
-  </si>
-  <si>
-    <t>empid</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>naveen</t>
-  </si>
-  <si>
-    <t>ravi</t>
-  </si>
-  <si>
-    <t>swami</t>
-  </si>
-  <si>
-    <t>rohit</t>
-  </si>
-  <si>
-    <t>escort</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>ayesha</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>male</t>
-  </si>
-  <si>
-    <t>female</t>
-  </si>
-  <si>
-    <t>per head cost</t>
-  </si>
-  <si>
-    <t>swetha</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
+  </numFmts>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -136,39 +68,138 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick"/>
+      <right style="thick"/>
+      <top style="thick"/>
+      <bottom style="thick"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -468,156 +499,317 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B994406-EF09-4D34-9E89-BED845F9C8E2}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.77734375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="9.109375" bestFit="1" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>trip ID</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>empid</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Shift type</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>escort</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>per head cost</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B2" s="2" t="n">
         <v>67678686676899</v>
       </c>
-      <c r="B2" s="1">
+      <c r="C2" s="1" t="n">
         <v>3456</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="1">
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>naveen</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B3" s="2" t="n">
         <v>67678686676899</v>
       </c>
-      <c r="B3" s="1">
+      <c r="C3" s="1" t="n">
         <v>3435</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1">
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>ravi</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B4" s="2" t="n">
         <v>67678686676899</v>
       </c>
-      <c r="B4" s="1">
+      <c r="C4" s="1" t="n">
         <v>8989</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="1">
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>swami</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n">
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B5" s="2" t="n">
         <v>77868689897897</v>
       </c>
-      <c r="B5" s="1">
+      <c r="C5" s="1" t="n">
         <v>7687</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>ayesha</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>morning</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B6" s="2" t="n">
         <v>68776768979880</v>
       </c>
-      <c r="B6" s="1">
+      <c r="C6" s="1" t="n">
         <v>7656</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="1">
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>rohit</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n">
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>68776760979880</v>
       </c>
-      <c r="B7" s="4">
+      <c r="C7" s="1" t="n">
         <v>4567</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="1">
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>swetha</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="n">
         <v>500</v>
       </c>
+    </row>
+    <row r="8">
+      <c r="G8" s="7" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H8" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A6:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>zdscb</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="C11:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="11">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>dfjb</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>